<commit_message>
Update NBVT test cases and boundaries for Lab4.1
</commit_message>
<xml_diff>
--- a/Test_Cases/Lab4_Normal_BVT.xlsx
+++ b/Test_Cases/Lab4_Normal_BVT.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="85">
   <si>
     <t>Test Strategy</t>
   </si>
@@ -100,7 +100,7 @@
     <t>Date:</t>
   </si>
   <si>
-    <t>16/7/2026</t>
+    <t>18/7/2026</t>
   </si>
   <si>
     <t>nom</t>
@@ -133,13 +133,13 @@
     <t>TC001</t>
   </si>
   <si>
-    <t>8 = Standard</t>
+    <t>7 = Standard</t>
   </si>
   <si>
     <t>TC002</t>
   </si>
   <si>
-    <t>6 = Standard</t>
+    <t>4 = Poor</t>
   </si>
   <si>
     <t>Score</t>
@@ -151,6 +151,9 @@
     <t>TC003</t>
   </si>
   <si>
+    <t>ThrownException</t>
+  </si>
+  <si>
     <t>12 - 15</t>
   </si>
   <si>
@@ -160,7 +163,7 @@
     <t>TC004</t>
   </si>
   <si>
-    <t>9 = Standard</t>
+    <t>8 = Standard</t>
   </si>
   <si>
     <t>6 - 11</t>
@@ -172,6 +175,9 @@
     <t>TC005</t>
   </si>
   <si>
+    <t>9 = Standard</t>
+  </si>
+  <si>
     <t>0 - 5</t>
   </si>
   <si>
@@ -181,7 +187,7 @@
     <t>TC006</t>
   </si>
   <si>
-    <t>12 = Excellent</t>
+    <t>11 = Standard</t>
   </si>
   <si>
     <t>TC007</t>
@@ -196,7 +202,7 @@
     <t>TC010</t>
   </si>
   <si>
-    <t>7 = Standard</t>
+    <t>5 = Poor</t>
   </si>
   <si>
     <t>TC011</t>
@@ -422,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -449,8 +455,11 @@
     <xf borderId="2" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -467,6 +476,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="6" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
@@ -485,13 +497,13 @@
     </xf>
     <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -921,9 +933,9 @@
       <c r="A6" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="11"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="7"/>
@@ -7747,25 +7759,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.0" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="15"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="16" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="17" t="s">
         <v>14</v>
       </c>
       <c r="N1" s="1"/>
@@ -7789,20 +7801,20 @@
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="17"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="8">
-        <v>24.0</v>
+      <c r="K2" s="19">
+        <v>-1.0</v>
       </c>
-      <c r="L2" s="8">
+      <c r="L2" s="6">
         <v>39.0</v>
       </c>
-      <c r="M2" s="8">
-        <v>11.0</v>
+      <c r="M2" s="19">
+        <v>-1.0</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -7819,16 +7831,16 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" ht="27.0" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="18" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="20" t="s">
         <v>18</v>
       </c>
       <c r="G3" s="8" t="s">
@@ -7839,14 +7851,14 @@
       <c r="J3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="8">
-        <v>25.0</v>
+      <c r="K3" s="19">
+        <v>0.0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="6">
         <v>40.0</v>
       </c>
-      <c r="M3" s="8">
-        <v>12.0</v>
+      <c r="M3" s="19">
+        <v>0.0</v>
       </c>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -7863,16 +7875,16 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" ht="27.0" customHeight="1">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="18" t="s">
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="20" t="s">
         <v>23</v>
       </c>
       <c r="G4" s="8" t="s">
@@ -7883,14 +7895,14 @@
       <c r="J4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="8">
-        <v>26.0</v>
+      <c r="K4" s="19">
+        <v>1.0</v>
       </c>
-      <c r="L4" s="8">
+      <c r="L4" s="6">
         <v>41.0</v>
       </c>
-      <c r="M4" s="8">
-        <v>13.0</v>
+      <c r="M4" s="19">
+        <v>1.0</v>
       </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -7907,17 +7919,17 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" ht="27.0" customHeight="1">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="18" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="10" t="s">
         <v>28</v>
       </c>
       <c r="H5" s="1"/>
@@ -7925,14 +7937,14 @@
       <c r="J5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="19">
         <v>43.0</v>
       </c>
-      <c r="L5" s="8">
+      <c r="L5" s="6">
         <v>130.0</v>
       </c>
-      <c r="M5" s="8">
-        <v>21.0</v>
+      <c r="M5" s="19">
+        <v>15.0</v>
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -7961,13 +7973,13 @@
       <c r="J6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="8">
-        <v>59.0</v>
+      <c r="K6" s="19">
+        <v>60.0</v>
       </c>
-      <c r="L6" s="8">
+      <c r="L6" s="6">
         <v>219.0</v>
       </c>
-      <c r="M6" s="8">
+      <c r="M6" s="19">
         <v>29.0</v>
       </c>
       <c r="N6" s="1"/>
@@ -7985,21 +7997,21 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="22" t="s">
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="25" t="s">
         <v>35</v>
       </c>
       <c r="H7" s="1"/>
@@ -8007,13 +8019,13 @@
       <c r="J7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="8">
-        <v>60.0</v>
+      <c r="K7" s="19">
+        <v>61.0</v>
       </c>
-      <c r="L7" s="8">
+      <c r="L7" s="6">
         <v>220.0</v>
       </c>
-      <c r="M7" s="8">
+      <c r="M7" s="19">
         <v>30.0</v>
       </c>
       <c r="N7" s="1"/>
@@ -8031,31 +8043,31 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" ht="27.0" customHeight="1">
-      <c r="A8" s="24"/>
-      <c r="B8" s="16" t="s">
+      <c r="A8" s="26"/>
+      <c r="B8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K8" s="8">
-        <v>61.0</v>
+      <c r="K8" s="19">
+        <v>62.0</v>
       </c>
-      <c r="L8" s="8">
+      <c r="L8" s="6">
         <v>221.0</v>
       </c>
-      <c r="M8" s="8">
+      <c r="M8" s="19">
         <v>31.0</v>
       </c>
       <c r="N8" s="1"/>
@@ -8082,16 +8094,16 @@
       <c r="C9" s="8">
         <v>130.0</v>
       </c>
-      <c r="D9" s="8">
-        <v>21.0</v>
+      <c r="D9" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="25" t="s">
+      <c r="G9" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H9" s="1"/>
@@ -8118,37 +8130,37 @@
       <c r="A10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="8">
-        <v>25.0</v>
+      <c r="B10" s="10">
+        <v>0.0</v>
       </c>
       <c r="C10" s="8">
         <v>130.0</v>
       </c>
-      <c r="D10" s="8">
-        <v>21.0</v>
+      <c r="D10" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="25" t="s">
+      <c r="F10" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="25" t="s">
+      <c r="G10" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
-      <c r="J10" s="16" t="s">
+      <c r="J10" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="K10" s="16" t="s">
+      <c r="K10" s="17" t="s">
         <v>42</v>
       </c>
       <c r="L10" s="1"/>
-      <c r="M10" s="26" t="s">
+      <c r="M10" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="N10" s="14"/>
+      <c r="N10" s="15"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -8166,38 +8178,38 @@
       <c r="A11" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="8">
-        <v>26.0</v>
+      <c r="B11" s="10">
+        <v>1.0</v>
       </c>
       <c r="C11" s="8">
         <v>130.0</v>
       </c>
-      <c r="D11" s="8">
-        <v>21.0</v>
+      <c r="D11" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="25" t="s">
+      <c r="G11" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="27">
-        <v>24.0</v>
+      <c r="J11" s="19">
+        <v>-1.0</v>
       </c>
-      <c r="K11" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="L11" s="15"/>
-      <c r="M11" s="6" t="s">
+      <c r="K11" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="N11" s="28" t="s">
+      <c r="L11" s="16"/>
+      <c r="M11" s="6" t="s">
         <v>46</v>
+      </c>
+      <c r="N11" s="30" t="s">
+        <v>47</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
@@ -8214,40 +8226,40 @@
     </row>
     <row r="12" ht="27.0" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
-      <c r="B12" s="8">
-        <v>59.0</v>
+      <c r="B12" s="10">
+        <v>60.0</v>
       </c>
       <c r="C12" s="8">
         <v>130.0</v>
       </c>
-      <c r="D12" s="8">
-        <v>21.0</v>
+      <c r="D12" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E12" s="25" t="s">
-        <v>48</v>
+      <c r="E12" s="27" t="s">
+        <v>49</v>
       </c>
-      <c r="F12" s="25" t="s">
-        <v>48</v>
+      <c r="F12" s="27" t="s">
+        <v>49</v>
       </c>
-      <c r="G12" s="25" t="s">
+      <c r="G12" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="6">
-        <v>25.0</v>
+      <c r="J12" s="19">
+        <v>0.0</v>
       </c>
-      <c r="K12" s="6">
-        <v>1.0</v>
+      <c r="K12" s="19">
+        <v>0.0</v>
       </c>
-      <c r="L12" s="15"/>
+      <c r="L12" s="16"/>
       <c r="M12" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
@@ -8264,40 +8276,40 @@
     </row>
     <row r="13" ht="27.0" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
-      <c r="B13" s="8">
-        <v>60.0</v>
+      <c r="B13" s="10">
+        <v>61.0</v>
       </c>
       <c r="C13" s="8">
         <v>130.0</v>
       </c>
-      <c r="D13" s="8">
-        <v>21.0</v>
+      <c r="D13" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E13" s="25" t="s">
-        <v>48</v>
+      <c r="E13" s="27" t="s">
+        <v>53</v>
       </c>
-      <c r="F13" s="25" t="s">
-        <v>48</v>
+      <c r="F13" s="27" t="s">
+        <v>53</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="6">
-        <v>26.0</v>
-      </c>
-      <c r="K13" s="27">
+      <c r="J13" s="19">
         <v>1.0</v>
       </c>
-      <c r="L13" s="15"/>
+      <c r="K13" s="19">
+        <v>0.0</v>
+      </c>
+      <c r="L13" s="16"/>
       <c r="M13" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
@@ -8314,7 +8326,7 @@
     </row>
     <row r="14" ht="27.0" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B14" s="8">
         <v>43.0</v>
@@ -8322,29 +8334,29 @@
       <c r="C14" s="8">
         <v>40.0</v>
       </c>
-      <c r="D14" s="8">
-        <v>21.0</v>
+      <c r="D14" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E14" s="25" t="s">
-        <v>55</v>
+      <c r="E14" s="27" t="s">
+        <v>57</v>
       </c>
-      <c r="F14" s="25" t="s">
-        <v>55</v>
+      <c r="F14" s="27" t="s">
+        <v>57</v>
       </c>
-      <c r="G14" s="25" t="s">
+      <c r="G14" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="6">
+      <c r="J14" s="19">
         <v>43.0</v>
       </c>
       <c r="K14" s="6">
         <v>3.0</v>
       </c>
-      <c r="L14" s="15"/>
+      <c r="L14" s="16"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="15"/>
+      <c r="N14" s="16"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
@@ -8360,7 +8372,7 @@
     </row>
     <row r="15" ht="27.0" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B15" s="8">
         <v>43.0</v>
@@ -8368,29 +8380,29 @@
       <c r="C15" s="8">
         <v>41.0</v>
       </c>
-      <c r="D15" s="8">
-        <v>21.0</v>
+      <c r="D15" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E15" s="25" t="s">
-        <v>55</v>
+      <c r="E15" s="27" t="s">
+        <v>57</v>
       </c>
-      <c r="F15" s="25" t="s">
-        <v>55</v>
+      <c r="F15" s="27" t="s">
+        <v>57</v>
       </c>
-      <c r="G15" s="25" t="s">
+      <c r="G15" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="6">
-        <v>59.0</v>
+      <c r="J15" s="19">
+        <v>60.0</v>
       </c>
       <c r="K15" s="6">
         <v>4.0</v>
       </c>
-      <c r="L15" s="15"/>
+      <c r="L15" s="16"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="15"/>
+      <c r="N15" s="16"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
@@ -8406,7 +8418,7 @@
     </row>
     <row r="16" ht="27.0" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B16" s="8">
         <v>43.0</v>
@@ -8414,29 +8426,29 @@
       <c r="C16" s="8">
         <v>219.0</v>
       </c>
-      <c r="D16" s="8">
-        <v>21.0</v>
+      <c r="D16" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="F16" s="25" t="s">
+      <c r="F16" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="6">
-        <v>60.0</v>
+      <c r="J16" s="19">
+        <v>61.0</v>
       </c>
-      <c r="K16" s="6">
-        <v>4.0</v>
+      <c r="K16" s="19">
+        <v>5.0</v>
       </c>
-      <c r="L16" s="15"/>
+      <c r="L16" s="16"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="15"/>
+      <c r="N16" s="16"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
@@ -8452,7 +8464,7 @@
     </row>
     <row r="17" ht="27.0" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B17" s="8">
         <v>43.0</v>
@@ -8460,29 +8472,29 @@
       <c r="C17" s="8">
         <v>220.0</v>
       </c>
-      <c r="D17" s="8">
-        <v>21.0</v>
+      <c r="D17" s="10">
+        <v>15.0</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="F17" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="25" t="s">
+      <c r="G17" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="6">
-        <v>61.0</v>
+      <c r="J17" s="19">
+        <v>62.0</v>
       </c>
       <c r="K17" s="6">
         <v>5.0</v>
       </c>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="15"/>
+      <c r="N17" s="16"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
@@ -8498,7 +8510,7 @@
     </row>
     <row r="18" ht="27.0" customHeight="1">
       <c r="A18" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B18" s="8">
         <v>43.0</v>
@@ -8506,24 +8518,24 @@
       <c r="C18" s="8">
         <v>130.0</v>
       </c>
-      <c r="D18" s="8">
-        <v>12.0</v>
+      <c r="D18" s="10">
+        <v>0.0</v>
       </c>
-      <c r="E18" s="25" t="s">
-        <v>60</v>
+      <c r="E18" s="27" t="s">
+        <v>62</v>
       </c>
-      <c r="F18" s="25" t="s">
-        <v>60</v>
+      <c r="F18" s="27" t="s">
+        <v>62</v>
       </c>
-      <c r="G18" s="25" t="s">
+      <c r="G18" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
@@ -8540,7 +8552,7 @@
     </row>
     <row r="19" ht="27.0" customHeight="1">
       <c r="A19" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B19" s="8">
         <v>43.0</v>
@@ -8548,24 +8560,24 @@
       <c r="C19" s="8">
         <v>130.0</v>
       </c>
-      <c r="D19" s="8">
-        <v>13.0</v>
+      <c r="D19" s="10">
+        <v>1.0</v>
       </c>
-      <c r="E19" s="25" t="s">
-        <v>60</v>
+      <c r="E19" s="27" t="s">
+        <v>62</v>
       </c>
-      <c r="F19" s="25" t="s">
-        <v>60</v>
+      <c r="F19" s="27" t="s">
+        <v>62</v>
       </c>
-      <c r="G19" s="25" t="s">
+      <c r="G19" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="16" t="s">
+      <c r="J19" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="K19" s="16" t="s">
+      <c r="K19" s="17" t="s">
         <v>42</v>
       </c>
       <c r="L19" s="1"/>
@@ -8586,7 +8598,7 @@
     </row>
     <row r="20" ht="27.0" customHeight="1">
       <c r="A20" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B20" s="8">
         <v>43.0</v>
@@ -8597,13 +8609,13 @@
       <c r="D20" s="8">
         <v>29.0</v>
       </c>
-      <c r="E20" s="25" t="s">
-        <v>48</v>
+      <c r="E20" s="28" t="s">
+        <v>53</v>
       </c>
-      <c r="F20" s="25" t="s">
-        <v>48</v>
+      <c r="F20" s="28" t="s">
+        <v>53</v>
       </c>
-      <c r="G20" s="25" t="s">
+      <c r="G20" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H20" s="1"/>
@@ -8611,8 +8623,8 @@
       <c r="J20" s="6">
         <v>39.0</v>
       </c>
-      <c r="K20" s="6">
-        <v>5.0</v>
+      <c r="K20" s="19" t="s">
+        <v>45</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
@@ -8632,7 +8644,7 @@
     </row>
     <row r="21" ht="27.0" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B21" s="8">
         <v>43.0</v>
@@ -8643,13 +8655,13 @@
       <c r="D21" s="8">
         <v>30.0</v>
       </c>
-      <c r="E21" s="25" t="s">
-        <v>48</v>
+      <c r="E21" s="28" t="s">
+        <v>53</v>
       </c>
-      <c r="F21" s="25" t="s">
-        <v>48</v>
+      <c r="F21" s="28" t="s">
+        <v>53</v>
       </c>
-      <c r="G21" s="25" t="s">
+      <c r="G21" s="28" t="s">
         <v>2</v>
       </c>
       <c r="H21" s="1"/>
@@ -8660,8 +8672,8 @@
       <c r="K21" s="6">
         <v>5.0</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
@@ -8692,8 +8704,8 @@
       <c r="K22" s="6">
         <v>5.0</v>
       </c>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -8724,8 +8736,8 @@
       <c r="K23" s="6">
         <v>1.0</v>
       </c>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
@@ -8756,8 +8768,8 @@
       <c r="K24" s="6">
         <v>1.0</v>
       </c>
-      <c r="L24" s="15"/>
-      <c r="M24" s="15"/>
+      <c r="L24" s="16"/>
+      <c r="M24" s="16"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
@@ -8788,8 +8800,8 @@
       <c r="K25" s="6">
         <v>1.0</v>
       </c>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
+      <c r="L25" s="16"/>
+      <c r="M25" s="16"/>
       <c r="N25" s="1"/>
       <c r="O25" s="1"/>
       <c r="P25" s="1"/>
@@ -8817,11 +8829,11 @@
       <c r="J26" s="6">
         <v>221.0</v>
       </c>
-      <c r="K26" s="6">
-        <v>1.0</v>
+      <c r="K26" s="19" t="s">
+        <v>45</v>
       </c>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -8846,7 +8858,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="15"/>
+      <c r="J27" s="16"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -8874,14 +8886,14 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="16" t="s">
+      <c r="J28" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="K28" s="16" t="s">
+      <c r="K28" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
       <c r="N28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
@@ -8906,11 +8918,11 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="6">
-        <v>11.0</v>
+      <c r="J29" s="19">
+        <v>-1.0</v>
       </c>
-      <c r="K29" s="6">
-        <v>1.0</v>
+      <c r="K29" s="19" t="s">
+        <v>45</v>
       </c>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -8938,11 +8950,11 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="6">
-        <v>12.0</v>
+      <c r="J30" s="19">
+        <v>0.0</v>
       </c>
-      <c r="K30" s="6">
-        <v>3.0</v>
+      <c r="K30" s="19">
+        <v>1.0</v>
       </c>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -8970,11 +8982,11 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="6">
-        <v>13.0</v>
+      <c r="J31" s="19">
+        <v>1.0</v>
       </c>
-      <c r="K31" s="6">
-        <v>3.0</v>
+      <c r="K31" s="19">
+        <v>1.0</v>
       </c>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -9002,11 +9014,11 @@
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="6">
-        <v>21.0</v>
+      <c r="J32" s="19">
+        <v>15.0</v>
       </c>
-      <c r="K32" s="6">
-        <v>4.0</v>
+      <c r="K32" s="19">
+        <v>3.0</v>
       </c>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -9034,7 +9046,7 @@
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="6">
+      <c r="J33" s="19">
         <v>29.0</v>
       </c>
       <c r="K33" s="6">
@@ -9066,7 +9078,7 @@
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="6">
+      <c r="J34" s="19">
         <v>30.0</v>
       </c>
       <c r="K34" s="6">
@@ -9098,7 +9110,7 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
       <c r="I35" s="1"/>
-      <c r="J35" s="6">
+      <c r="J35" s="19">
         <v>31.0</v>
       </c>
       <c r="K35" s="6">
@@ -15525,25 +15537,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="27.0" customHeight="1">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="15"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="16" t="s">
+      <c r="J1" s="16"/>
+      <c r="K1" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="17" t="s">
         <v>14</v>
       </c>
       <c r="N1" s="1"/>
@@ -15567,15 +15579,15 @@
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="17"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
@@ -15591,16 +15603,16 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" ht="27.0" customHeight="1">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>64</v>
+      <c r="B3" s="21" t="s">
+        <v>66</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="18" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="20" t="s">
         <v>18</v>
       </c>
       <c r="G3" s="8"/>
@@ -15609,9 +15621,9 @@
       <c r="J3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="29"/>
-      <c r="L3" s="29"/>
-      <c r="M3" s="29"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
@@ -15627,16 +15639,16 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" ht="27.0" customHeight="1">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="19" t="s">
-        <v>65</v>
+      <c r="B4" s="21" t="s">
+        <v>67</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="18" t="s">
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="20" t="s">
         <v>23</v>
       </c>
       <c r="G4" s="8"/>
@@ -15645,9 +15657,9 @@
       <c r="J4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="29"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
@@ -15663,14 +15675,14 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" ht="27.0" customHeight="1">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="18" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="20" t="s">
         <v>27</v>
       </c>
       <c r="G5" s="8"/>
@@ -15679,9 +15691,9 @@
       <c r="J5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -15709,9 +15721,9 @@
       <c r="J6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="29"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="31"/>
+      <c r="M6" s="31"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
@@ -15727,21 +15739,21 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" ht="24.75" customHeight="1">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="22" t="s">
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="25" t="s">
         <v>35</v>
       </c>
       <c r="H7" s="1"/>
@@ -15749,9 +15761,9 @@
       <c r="J7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="29"/>
-      <c r="L7" s="29"/>
-      <c r="M7" s="29"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="31"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
@@ -15767,27 +15779,27 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" ht="27.0" customHeight="1">
-      <c r="A8" s="24"/>
-      <c r="B8" s="16" t="s">
+      <c r="A8" s="26"/>
+      <c r="B8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="29"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31"/>
+      <c r="M8" s="31"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -15894,7 +15906,7 @@
     </row>
     <row r="12" ht="27.0" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -15904,10 +15916,10 @@
       <c r="G12" s="8"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
@@ -15924,7 +15936,7 @@
     </row>
     <row r="13" ht="27.0" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -15934,10 +15946,10 @@
       <c r="G13" s="8"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="15"/>
-      <c r="M13" s="15"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="16"/>
+      <c r="M13" s="16"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
@@ -15954,7 +15966,7 @@
     </row>
     <row r="14" ht="27.0" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -15964,10 +15976,10 @@
       <c r="G14" s="8"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
@@ -15984,7 +15996,7 @@
     </row>
     <row r="15" ht="27.0" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -15994,10 +16006,10 @@
       <c r="G15" s="8"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
@@ -16014,7 +16026,7 @@
     </row>
     <row r="16" ht="27.0" customHeight="1">
       <c r="A16" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -16024,10 +16036,10 @@
       <c r="G16" s="8"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
@@ -16044,7 +16056,7 @@
     </row>
     <row r="17" ht="27.0" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -16054,10 +16066,10 @@
       <c r="G17" s="8"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -16074,7 +16086,7 @@
     </row>
     <row r="18" ht="27.0" customHeight="1">
       <c r="A18" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -16084,10 +16096,10 @@
       <c r="G18" s="8"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
@@ -16104,7 +16116,7 @@
     </row>
     <row r="19" ht="27.0" customHeight="1">
       <c r="A19" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -16114,10 +16126,10 @@
       <c r="G19" s="8"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="15"/>
-      <c r="M19" s="15"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
@@ -16134,7 +16146,7 @@
     </row>
     <row r="20" ht="27.0" customHeight="1">
       <c r="A20" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -16144,7 +16156,7 @@
       <c r="G20" s="8"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="15"/>
+      <c r="J20" s="16"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
@@ -16164,7 +16176,7 @@
     </row>
     <row r="21" ht="27.0" customHeight="1">
       <c r="A21" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -16174,10 +16186,10 @@
       <c r="G21" s="8"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
@@ -16194,7 +16206,7 @@
     </row>
     <row r="22" ht="27.0" customHeight="1">
       <c r="A22" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -16204,10 +16216,10 @@
       <c r="G22" s="8"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
@@ -16224,7 +16236,7 @@
     </row>
     <row r="23" ht="27.0" customHeight="1">
       <c r="A23" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -16234,10 +16246,10 @@
       <c r="G23" s="8"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="15"/>
-      <c r="M23" s="15"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
@@ -16254,7 +16266,7 @@
     </row>
     <row r="24" ht="27.0" customHeight="1">
       <c r="A24" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -16284,7 +16296,7 @@
     </row>
     <row r="25" ht="27.0" customHeight="1">
       <c r="A25" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -16314,7 +16326,7 @@
     </row>
     <row r="26" ht="27.0" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -16324,10 +16336,10 @@
       <c r="G26" s="8"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
+      <c r="J26" s="16"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
       <c r="N26" s="1"/>
       <c r="O26" s="1"/>
       <c r="P26" s="1"/>
@@ -16344,7 +16356,7 @@
     </row>
     <row r="27" ht="27.0" customHeight="1">
       <c r="A27" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -16354,10 +16366,10 @@
       <c r="G27" s="8"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="15"/>
-      <c r="K27" s="15"/>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
       <c r="N27" s="1"/>
       <c r="O27" s="1"/>
       <c r="P27" s="1"/>
@@ -16382,10 +16394,10 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="16"/>
+      <c r="L28" s="16"/>
+      <c r="M28" s="16"/>
       <c r="N28" s="1"/>
       <c r="O28" s="1"/>
       <c r="P28" s="1"/>
@@ -22804,38 +22816,38 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" ht="27.0" customHeight="1">
-      <c r="A2" s="30" t="s">
-        <v>72</v>
-      </c>
-      <c r="B2" s="30" t="s">
-        <v>73</v>
-      </c>
-      <c r="C2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="B2" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="C2" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="F2" s="30" t="s">
+      <c r="D2" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="G2" s="30" t="s">
+      <c r="E2" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="F2" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="G2" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="30" t="s">
+      <c r="H2" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="K2" s="30" t="s">
+      <c r="I2" s="32" t="s">
         <v>82</v>
+      </c>
+      <c r="J2" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="K2" s="32" t="s">
+        <v>84</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -22854,19 +22866,19 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" ht="27.0" customHeight="1">
-      <c r="A3" s="32">
+      <c r="A3" s="34">
         <v>1.0</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>

</xml_diff>